<commit_message>
update product field and asset form
</commit_message>
<xml_diff>
--- a/wwwroot/assets/doc_form/assets_upload_format.xlsx
+++ b/wwwroot/assets/doc_form/assets_upload_format.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\iHishab\iHishab\wwwroot\assets\doc_form\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C0145F7-77AD-481C-9749-DD6CA0BF095A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F898A74-3297-4ACF-9FE2-68B15DBA1225}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{77913F84-C404-4304-BA6F-166839364020}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{77913F84-C404-4304-BA6F-166839364020}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>AssetName</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>AssetLocation</t>
+  </si>
+  <si>
+    <t>Country of Origin</t>
   </si>
 </sst>
 </file>
@@ -432,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E604C800-FE24-48A3-A3EF-9FFD3F151312}">
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
@@ -442,15 +445,15 @@
     <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -473,25 +476,29 @@
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>